<commit_message>
redesign some shit on wheel and other stuff
</commit_message>
<xml_diff>
--- a/_MK-1_/NeoSumec_MK-1_MECH.xlsx
+++ b/_MK-1_/NeoSumec_MK-1_MECH.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zak\GitHub\NeoSumec-MiniSumo-MECH\_MK-1_\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F0E05EF-3039-480D-8CEA-6BC02AEA335C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE3FA6C5-DAC3-444C-9063-8CB4B5647FDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{E70E74EA-06C0-433E-BC4D-5A3409939100}"/>
   </bookViews>
@@ -93,20 +93,41 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.14999847407452621"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -122,7 +143,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -463,9 +484,9 @@
   <dimension ref="A1:D5"/>
   <sheetFormatPr defaultColWidth="4.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.109375" style="1" customWidth="1"/>
-    <col min="2" max="2" width="5.44140625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="6.6640625" style="1" customWidth="1"/>
+    <col min="1" max="1" width="12.33203125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="6.109375" style="1" customWidth="1"/>
+    <col min="3" max="3" width="7.21875" style="1" customWidth="1"/>
     <col min="4" max="16384" width="4.44140625" style="1"/>
   </cols>
   <sheetData>

</xml_diff>

<commit_message>
Some rework and adjust tolerance
</commit_message>
<xml_diff>
--- a/_MK-1_/NeoSumec_MK-1_MECH.xlsx
+++ b/_MK-1_/NeoSumec_MK-1_MECH.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zak\GitHub\NeoSumec-MiniSumo-MECH\_MK-1_\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE3FA6C5-DAC3-444C-9063-8CB4B5647FDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75BAAB4C-2363-4509-92B0-D74EFD55E57F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{E70E74EA-06C0-433E-BC4D-5A3409939100}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="15">
   <si>
     <t>Name</t>
   </si>
@@ -47,19 +47,40 @@
     <t>Link</t>
   </si>
   <si>
-    <t xml:space="preserve">M3 Din 934 </t>
-  </si>
-  <si>
     <t>M3x25 Torx</t>
   </si>
   <si>
     <t>M3x20 Torx</t>
   </si>
   <si>
-    <t>M3x45 Hex</t>
-  </si>
-  <si>
     <t>?</t>
+  </si>
+  <si>
+    <t>M3x16 Torx</t>
+  </si>
+  <si>
+    <t>M3x0,5</t>
+  </si>
+  <si>
+    <t>Comment</t>
+  </si>
+  <si>
+    <t>Matice</t>
+  </si>
+  <si>
+    <t>Motor vzad</t>
+  </si>
+  <si>
+    <t>Motor vpřed</t>
+  </si>
+  <si>
+    <t>Osa rotace</t>
+  </si>
+  <si>
+    <t>M3x0.3</t>
+  </si>
+  <si>
+    <t>Matice čtyřhran</t>
   </si>
 </sst>
 </file>
@@ -481,16 +502,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C58A2579-B6B4-43B1-AA5E-44312C298E05}">
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr defaultColWidth="4.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.33203125" style="1" customWidth="1"/>
     <col min="2" max="2" width="6.109375" style="1" customWidth="1"/>
     <col min="3" max="3" width="7.21875" style="1" customWidth="1"/>
-    <col min="4" max="16384" width="4.44140625" style="1"/>
+    <col min="4" max="4" width="15" style="1" customWidth="1"/>
+    <col min="5" max="16384" width="4.44140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -500,10 +522,13 @@
       <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
+      <c r="D1" s="3" t="s">
+        <v>8</v>
+      </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="B2" s="1">
         <v>4</v>
@@ -511,55 +536,73 @@
       <c r="C2" s="2" t="s">
         <v>2</v>
       </c>
+      <c r="D2" s="1" t="s">
+        <v>9</v>
+      </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" s="1">
+        <v>2</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="1">
-        <v>2</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>7</v>
+      <c r="B5" s="1">
+        <v>2</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4" s="1">
-        <v>2</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A5" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B5" s="1">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="1">
         <v>1</v>
       </c>
-      <c r="C5" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>7</v>
+      <c r="C6" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>12</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="C2" r:id="rId1" xr:uid="{517062B2-C385-4292-8D30-9A915CC87D3F}"/>
-    <hyperlink ref="C4" r:id="rId2" xr:uid="{DF4E92D8-3D63-4001-A402-5388A1064A13}"/>
-    <hyperlink ref="C3" r:id="rId3" xr:uid="{929E184F-7BEF-406E-BCCA-C18D00D67E2D}"/>
-    <hyperlink ref="C5" r:id="rId4" xr:uid="{2A5722CB-6D09-4A6B-8DEE-E4D0759E4F18}"/>
+    <hyperlink ref="C5" r:id="rId2" xr:uid="{DF4E92D8-3D63-4001-A402-5388A1064A13}"/>
+    <hyperlink ref="C4" r:id="rId3" xr:uid="{CD317AC6-70D6-4FAA-82DC-062D351DD800}"/>
+    <hyperlink ref="C3" r:id="rId4" xr:uid="{9C5AFEAA-C950-4E19-8D53-8DAA31C707E1}"/>
+    <hyperlink ref="C6" r:id="rId5" xr:uid="{7454B801-582F-42C8-9E89-E8EDF2B0335C}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>